<commit_message>
Updates psgr-LDV exponent & shareweights to align with historic data & projections from ICCT
</commit_message>
<xml_diff>
--- a/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
+++ b/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\trans\TTLE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\TTLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38156F0C-A178-4103-B28F-F0C9E7C7D60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60338155-4D1D-4A3C-91F5-32B7D8C9F62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="855" yWindow="1830" windowWidth="26040" windowHeight="14730" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -767,18 +767,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="60">
     <cellStyle name="20% - Accent1" xfId="33" builtinId="30" customBuiltin="1"/>
@@ -886,9 +883,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -926,9 +923,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -961,26 +958,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1013,26 +993,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1206,7 +1169,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="45.453125" customWidth="1"/>
@@ -1221,199 +1184,52 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="2"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B11" s="2"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="2"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B16" s="2"/>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B18" s="2"/>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="25" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="2:2" s="2" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B30" s="2"/>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B31" s="2"/>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B32" s="2"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B33" s="2"/>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B34" s="2"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B35" s="2"/>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B36" s="2"/>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B37" s="2"/>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B38" s="2"/>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B39" s="2"/>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B40" s="2"/>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B41" s="2"/>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B42" s="2"/>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B43" s="2"/>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B44" s="2"/>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B45" s="2"/>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B46" s="2"/>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B47" s="2"/>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B48" s="2"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B49" s="2"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B50" s="2"/>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" s="1"/>
-      <c r="B51" s="2"/>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B52" s="2"/>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B53" s="2"/>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B54" s="2"/>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B55" s="2"/>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B56" s="2"/>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B57" s="2"/>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B58" s="2"/>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B59" s="2"/>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B60" s="2"/>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B61" s="2"/>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B62" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1435,13 +1251,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1449,10 +1265,10 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>-3</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="B2">
+        <v>-17.27</v>
+      </c>
+      <c r="C2">
         <v>-3</v>
       </c>
     </row>
@@ -1460,10 +1276,10 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3">
         <v>-3</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3">
         <v>-3</v>
       </c>
     </row>
@@ -1471,10 +1287,10 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4">
         <v>-3</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4">
         <v>-3</v>
       </c>
     </row>
@@ -1482,10 +1298,10 @@
       <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>-3</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>-3</v>
       </c>
     </row>
@@ -1493,10 +1309,10 @@
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>-3</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>-3</v>
       </c>
     </row>
@@ -1504,10 +1320,10 @@
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <v>-3</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7">
         <v>-3</v>
       </c>
     </row>
@@ -1517,6 +1333,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1660,7 +1482,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1669,20 +1491,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBF47025-38FC-4D4C-A172-57EF19919DA6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EE2417C-9996-4510-9140-E726E730908D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF0E423-9D38-426D-8974-49181EF85CAD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBF47025-38FC-4D4C-A172-57EF19919DA6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EE2417C-9996-4510-9140-E726E730908D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF0E423-9D38-426D-8974-49181EF85CAD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
TTS/TTLE update to use Marklines historical data, still align with ICCT future sales
</commit_message>
<xml_diff>
--- a/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
+++ b/InputData/trans/TTLE/Transportation Technology Logit Exponents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\TTLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60338155-4D1D-4A3C-91F5-32B7D8C9F62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C493D1C-A248-4271-B070-6073FCB4878E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="855" yWindow="1830" windowWidth="26040" windowHeight="14730" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -1170,17 +1170,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="45.453125" customWidth="1"/>
+    <col min="2" max="2" width="45.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1188,47 +1188,47 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
     </row>
   </sheetData>
@@ -1243,14 +1243,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1261,18 +1261,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2">
-        <v>-17.27</v>
+        <v>-13</v>
       </c>
       <c r="C2">
         <v>-3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1339,6 +1339,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1482,15 +1491,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7EE2417C-9996-4510-9140-E726E730908D}">
   <ds:schemaRefs>
@@ -1501,6 +1501,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF0E423-9D38-426D-8974-49181EF85CAD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBF47025-38FC-4D4C-A172-57EF19919DA6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1516,12 +1524,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF0E423-9D38-426D-8974-49181EF85CAD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>